<commit_message>
test(spi-worker): default-tenant 配置 Excel 加 SPI 四类 job
docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
的 job_definition sheet 追加 spi_shell/sql/stored_proc/http_demo 四行(job_type=SPI,
worker_group=spi,default_params 对齐 platform_seed.sql 的执行器协议),让租户配置包 Excel
导入路径也覆盖 SPI 原子任务,与种子脚本一致。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2241,6 +2241,338 @@
       <c r="T4" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe MIXED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>default-tenant</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>spi_shell_demo</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SPI Shell Demo</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SPI</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>spi_queue</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>spi</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>always_open</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>EXPONENTIAL</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>300</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>{"taskType":"shell","command":"/bin/echo","args":["hello-from-spi"]}</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>SPI demo - SPI Shell Demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>default-tenant</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>spi_sql_demo</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SPI SQL Demo</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SPI</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>spi_queue</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>spi</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>always_open</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>EXPONENTIAL</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
+        <v>300</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>{"taskType":"sql","sql":"SELECT 1"}</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>SPI demo - SPI SQL Demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>default-tenant</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>spi_stored_proc_demo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SPI Stored Proc Demo</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SPI</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>spi_queue</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>spi</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>always_open</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>EXPONENTIAL</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>300</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>{"taskType":"stored_proc","procedureName":"batch.refresh_metrics"}</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>SPI demo - SPI Stored Proc Demo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>default-tenant</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>spi_http_demo</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SPI HTTP Demo</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SPI</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>spi_queue</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>spi</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>always_open</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>EXPONENTIAL</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" t="n">
+        <v>300</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>STATIC</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>{"taskType":"http","url":"https://example.internal/health","method":"GET"}</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>SPI demo - SPI HTTP Demo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: harden strict and sim validation fixtures
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2009,6 +2009,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2087,6 +2092,11 @@
           <t>P2 seed aligned - Probe PIPELINE</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2165,6 +2175,11 @@
           <t>P2 seed aligned - Probe GATEWAY</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2243,6 +2258,11 @@
           <t>P2 seed aligned - Probe MIXED</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2326,6 +2346,11 @@
           <t>SPI demo - SPI Shell Demo</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2409,6 +2434,11 @@
           <t>SPI demo - SPI SQL Demo</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2492,6 +2522,11 @@
           <t>SPI demo - SPI Stored Proc Demo</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2573,6 +2608,11 @@
       <c r="T8" t="inlineStr">
         <is>
           <t>SPI demo - SPI HTTP Demo</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: harden strict and sim validation fixtures (#642)
Co-authored-by: idengzhao <40328852+idengzhao@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2009,6 +2009,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2087,6 +2092,11 @@
           <t>P2 seed aligned - Probe PIPELINE</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2165,6 +2175,11 @@
           <t>P2 seed aligned - Probe GATEWAY</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2243,6 +2258,11 @@
           <t>P2 seed aligned - Probe MIXED</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2326,6 +2346,11 @@
           <t>SPI demo - SPI Shell Demo</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2409,6 +2434,11 @@
           <t>SPI demo - SPI SQL Demo</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2492,6 +2522,11 @@
           <t>SPI demo - SPI Stored Proc Demo</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2573,6 +2608,11 @@
       <c r="T8" t="inlineStr">
         <is>
           <t>SPI demo - SPI HTTP Demo</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sim): align tenant package Excel fixtures
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,62 +1956,72 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>depends_on_job_code</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>calendar_code</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>window_code</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>retry_policy</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>retry_max_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>timeout_seconds</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>shard_strategy</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>execution_handler</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>param_schema</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>default_params</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>execution_mode</t>
         </is>
       </c>
     </row>
@@ -2051,50 +2061,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
       <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>14400</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe PIPELINE</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -2134,50 +2144,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>14400</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe GATEWAY</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -2217,402 +2227,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>14400</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe MIXED</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>spi_shell_demo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SPI Shell Demo</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>300</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{"taskType":"shell","command":"/bin/echo","args":["hello-from-spi"]}</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI Shell Demo</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>spi_sql_demo</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SPI SQL Demo</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>300</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>{"taskType":"sql","sql":"SELECT 1"}</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI SQL Demo</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>spi_stored_proc_demo</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SPI Stored Proc Demo</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>300</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>{"taskType":"stored_proc","procedureName":"batch.refresh_metrics"}</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI Stored Proc Demo</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>spi_http_demo</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SPI HTTP Demo</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>300</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>{"taskType":"http","url":"https://example.internal/health","method":"GET"}</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI HTTP Demo</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(orchestrator,sim): repair worker fallback and tenant package fixtures (#979)
* fix(orchestrator): fall back past inactive tenant worker

* fix(sim): align tenant package Excel fixtures

---------

Co-authored-by: Dengchao <tfys9544@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,62 +1956,72 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>depends_on_job_code</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>calendar_code</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>window_code</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>retry_policy</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>retry_max_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>timeout_seconds</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>shard_strategy</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>execution_handler</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>param_schema</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>default_params</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>execution_mode</t>
         </is>
       </c>
     </row>
@@ -2051,50 +2061,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
       <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>14400</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe PIPELINE</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -2134,50 +2144,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
       <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
         <v>14400</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe GATEWAY</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>
@@ -2217,402 +2227,50 @@
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>always_open</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
       <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
         <v>14400</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>P2 seed aligned - Probe MIXED</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>spi_shell_demo</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SPI Shell Demo</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" t="n">
-        <v>300</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>{"taskType":"shell","command":"/bin/echo","args":["hello-from-spi"]}</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI Shell Demo</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>spi_sql_demo</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SPI SQL Demo</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>300</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>{"taskType":"sql","sql":"SELECT 1"}</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI SQL Demo</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>spi_stored_proc_demo</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SPI Stored Proc Demo</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
-        <v>300</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>{"taskType":"stored_proc","procedureName":"batch.refresh_metrics"}</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI Stored Proc Demo</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>FULL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>default-tenant</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>spi_http_demo</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SPI HTTP Demo</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>spi_queue</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>spi</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>always_open</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>EXPONENTIAL</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="n">
-        <v>300</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>STATIC</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>{"taskType":"http","url":"https://example.internal/health","method":"GET"}</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>SPI demo - SPI HTTP Demo</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>FULL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(import): align sim fixture import config
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
test(import): align sim fixture import config (#984)
Co-authored-by: Dengchao <tfys9544@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
+++ b/docs/test-data/test-full-coverage-import-suite/default-tenant-config-package-test.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>